<commit_message>
commit "complete framework updates"
</commit_message>
<xml_diff>
--- a/Ecommerce.BITM.SwagLabs/src/test/resources/TestData.xlsx
+++ b/Ecommerce.BITM.SwagLabs/src/test/resources/TestData.xlsx
@@ -3,18 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{B906CAC1-197B-47CD-82B9-77043A810065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{02727C11-B337-4A0E-83F4-A371C8869718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{CC12B2A3-8707-4673-8865-24C19DBF021D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{CC12B2A3-8707-4673-8865-24C19DBF021D}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="3" r:id="rId1"/>
     <sheet name="InvalidLogin" sheetId="1" r:id="rId2"/>
     <sheet name="CheckoutDetails" sheetId="2" r:id="rId3"/>
-    <sheet name="BoundaryLoginData" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A3:N9"/>
+  <oleSize ref="A1:Q8"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
   <si>
     <t>username</t>
   </si>
@@ -68,9 +67,6 @@
     <t>swati@123</t>
   </si>
   <si>
-    <t>standard_user</t>
-  </si>
-  <si>
     <t>performance_glitch_user</t>
   </si>
   <si>
@@ -78,9 +74,6 @@
   </si>
   <si>
     <t>visual_user</t>
-  </si>
-  <si>
-    <t>Password</t>
   </si>
 </sst>
 </file>
@@ -457,14 +450,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C10263CD-5853-4B6E-9425-1039EE20CDE9}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.5546875" customWidth="1"/>
     <col min="2" max="2" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -472,9 +465,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>4</v>
@@ -482,7 +475,7 @@
     </row>
     <row r="3" spans="1:2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>4</v>
@@ -504,15 +497,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
+    <row r="6" spans="1:2" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="7" spans="1:2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:2" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -631,36 +618,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0214FE73-4799-496F-A3CF-C21B97B68106}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.77734375" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>